<commit_message>
Integrate enhanced checkin mediation workflow
</commit_message>
<xml_diff>
--- a/data/example/checkin/glycemic/eps_chat_history.xlsx
+++ b/data/example/checkin/glycemic/eps_chat_history.xlsx
@@ -474,14 +474,14 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>今天完成了25分钟快走和拉伸。</t>
+          <t>今天餐后散步22分钟，空腹血糖感觉比前几天稳定一些。</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-11 19:07</t>
+          <t>2026-03-11 12:07</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -496,14 +496,14 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>@Yara #exercise_feedback 已记录，今天第1次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Yara #exercise_feedback 做得不错，你这周的执行比较稳定。可以尝试把晚餐后活动固定下来，关注空腹和餐后血糖变化。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-11 19:10</t>
+          <t>2026-03-11 15:10</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -518,7 +518,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>@Yara #exercise_feedback 已记录，今天第2次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Yara #exercise_feedback 今天反馈重点是控糖连续性。建议晚餐主食再略减一些，并保持饭后快走，你有明显进步。</t>
         </is>
       </c>
     </row>
@@ -540,7 +540,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>收到，谢谢老师，我明天继续打卡。</t>
+          <t>收到，我会继续按这个节奏控糖。</t>
         </is>
       </c>
     </row>
@@ -562,14 +562,14 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>今天完成了30分钟快走和拉伸。</t>
+          <t>上午快走后记录了血糖，下午又做了轻度力量训练。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-03-12 19:25</t>
+          <t>2026-03-12 13:25</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -584,14 +584,14 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>@Zoe #exercise_feedback 已记录，今天第1次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Zoe #exercise_feedback 今天反馈重点是控糖连续性。建议晚餐主食再略减一些，并保持饭后快走，你有明显进步。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-03-12 19:28</t>
+          <t>2026-03-12 16:28</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -606,7 +606,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>@Zoe #exercise_feedback 已记录，今天第2次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Zoe #exercise_feedback 很棒，结合你目前的情况，推荐继续中等强度步行并记录空腹血糖，注意作息规律。</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>@Zoe #exercise_feedback 已记录，今天第3次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Zoe #exercise_feedback 很好。根据你最近的血糖记录，建议餐后再步行10到15分钟，继续保持控糖节奏。</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>收到，谢谢老师，我明天继续打卡。</t>
+          <t>好的，我明天把饭后步行时间再延长一点。</t>
         </is>
       </c>
     </row>
@@ -672,14 +672,14 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>今天完成了35分钟快走和拉伸。</t>
+          <t>今天控制了晚餐，总步数大概6150步，餐后活动也完成了。</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-03-13 19:46</t>
+          <t>2026-03-13 11:46</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -694,14 +694,14 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>@Aaron #exercise_feedback 已记录，今天第1次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Aaron #exercise_feedback 很棒，结合你目前的情况，推荐继续中等强度步行并记录空腹血糖，注意作息规律。</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-03-13 19:49</t>
+          <t>2026-03-13 14:49</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -716,14 +716,14 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>@Aaron #exercise_feedback 已记录，今天第2次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Aaron #exercise_feedback 很好。根据你最近的血糖记录，建议餐后再步行10到15分钟，继续保持控糖节奏。</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-03-13 19:52</t>
+          <t>2026-03-13 17:52</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>@Aaron #exercise_feedback 已记录，今天第3次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Aaron #exercise_feedback 做得不错，你这周的执行比较稳定。可以尝试把晚餐后活动固定下来，关注空腹和餐后血糖变化。</t>
         </is>
       </c>
     </row>
@@ -760,7 +760,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>收到，谢谢老师，我明天继续打卡。</t>
+          <t>明白了，我会继续记录空腹和餐后情况。</t>
         </is>
       </c>
     </row>
@@ -782,14 +782,14 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>今天完成了40分钟快走和拉伸。</t>
+          <t>今天按照计划运动，餐后没有吃零食，准备继续观察空腹血糖。</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-03-14 19:07</t>
+          <t>2026-03-14 12:07</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -804,14 +804,14 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>@Blake #exercise_feedback 已记录，今天第1次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Blake #exercise_feedback 很好。根据你最近的血糖记录，建议餐后再步行10到15分钟，继续保持控糖节奏。</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-03-14 19:10</t>
+          <t>2026-03-14 15:10</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -826,14 +826,14 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>@Blake #exercise_feedback 已记录，今天第2次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Blake #exercise_feedback 做得不错，你这周的执行比较稳定。可以尝试把晚餐后活动固定下来，关注空腹和餐后血糖变化。</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-03-14 19:13</t>
+          <t>2026-03-14 18:13</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -848,14 +848,14 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>@Blake #exercise_feedback 已记录，今天第3次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Blake #exercise_feedback 今天反馈重点是控糖连续性。建议晚餐主食再略减一些，并保持饭后快走，你有明显进步。</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-03-14 19:16</t>
+          <t>2026-03-14 21:16</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>@Blake #exercise_feedback 已记录，今天第4次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Blake #exercise_feedback 很棒，结合你目前的情况，推荐继续中等强度步行并记录空腹血糖，注意作息规律。</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>收到，谢谢老师，我明天继续打卡。</t>
+          <t>收到，我会继续按这个节奏控糖。</t>
         </is>
       </c>
     </row>
@@ -914,14 +914,14 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>今天完成了45分钟快走和拉伸。</t>
+          <t>今天餐后散步38分钟，空腹血糖感觉比前几天稳定一些。</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-03-15 19:31</t>
+          <t>2026-03-15 13:31</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -936,14 +936,14 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>@Carter #exercise_feedback 已记录，今天第1次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Carter #exercise_feedback 做得不错，你这周的执行比较稳定。可以尝试把晚餐后活动固定下来，关注空腹和餐后血糖变化。</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-03-15 19:34</t>
+          <t>2026-03-15 16:34</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -958,7 +958,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>@Carter #exercise_feedback 已记录，今天第2次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Carter #exercise_feedback 今天反馈重点是控糖连续性。建议晚餐主食再略减一些，并保持饭后快走，你有明显进步。</t>
         </is>
       </c>
     </row>
@@ -980,7 +980,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>收到，谢谢老师，我明天继续打卡。</t>
+          <t>好的，我明天把饭后步行时间再延长一点。</t>
         </is>
       </c>
     </row>
@@ -1002,14 +1002,14 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>今天完成了50分钟快走和拉伸。</t>
+          <t>上午快走后记录了血糖，下午又做了轻度力量训练。</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-03-16 19:49</t>
+          <t>2026-03-16 11:49</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1024,14 +1024,14 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>@Derek #exercise_feedback 已记录，今天第1次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Derek #exercise_feedback 今天反馈重点是控糖连续性。建议晚餐主食再略减一些，并保持饭后快走，你有明显进步。</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-03-16 19:52</t>
+          <t>2026-03-16 14:52</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1046,14 +1046,14 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>@Derek #exercise_feedback 已记录，今天第2次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Derek #exercise_feedback 很棒，结合你目前的情况，推荐继续中等强度步行并记录空腹血糖，注意作息规律。</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-03-16 19:55</t>
+          <t>2026-03-16 17:55</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1068,14 +1068,14 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>@Derek #exercise_feedback 已记录，今天第3次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Derek #exercise_feedback 很好。根据你最近的血糖记录，建议餐后再步行10到15分钟，继续保持控糖节奏。</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-03-16 19:58</t>
+          <t>2026-03-16 20:58</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>@Derek #exercise_feedback 已记录，今天第4次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Derek #exercise_feedback 做得不错，你这周的执行比较稳定。可以尝试把晚餐后活动固定下来，关注空腹和餐后血糖变化。</t>
         </is>
       </c>
     </row>
@@ -1112,7 +1112,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>收到，谢谢老师，我明天继续打卡。</t>
+          <t>明白了，我会继续记录空腹和餐后情况。</t>
         </is>
       </c>
     </row>
@@ -1134,14 +1134,14 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>今天完成了55分钟快走和拉伸。</t>
+          <t>今天控制了晚餐，总步数大概8750步，餐后活动也完成了。</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-03-17 19:13</t>
+          <t>2026-03-17 12:13</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1156,14 +1156,14 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>@Ethan #exercise_feedback 已记录，今天第1次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Ethan #exercise_feedback 很棒，结合你目前的情况，推荐继续中等强度步行并记录空腹血糖，注意作息规律。</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-03-17 19:16</t>
+          <t>2026-03-17 15:16</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1178,14 +1178,14 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>@Ethan #exercise_feedback 已记录，今天第2次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Ethan #exercise_feedback 很好。根据你最近的血糖记录，建议餐后再步行10到15分钟，继续保持控糖节奏。</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-03-17 19:19</t>
+          <t>2026-03-17 18:19</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>@Ethan #exercise_feedback 已记录，今天第3次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Ethan #exercise_feedback 做得不错，你这周的执行比较稳定。可以尝试把晚餐后活动固定下来，关注空腹和餐后血糖变化。</t>
         </is>
       </c>
     </row>
@@ -1222,7 +1222,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>收到，谢谢老师，我明天继续打卡。</t>
+          <t>收到，我会继续按这个节奏控糖。</t>
         </is>
       </c>
     </row>
@@ -1244,14 +1244,14 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>今天完成了60分钟快走和拉伸。</t>
+          <t>今天按照计划运动，餐后没有吃零食，准备继续观察空腹血糖。</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-03-18 19:34</t>
+          <t>2026-03-18 13:34</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1266,14 +1266,14 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>@Felix #exercise_feedback 已记录，今天第1次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Felix #exercise_feedback 很好。根据你最近的血糖记录，建议餐后再步行10到15分钟，继续保持控糖节奏。</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-03-18 19:37</t>
+          <t>2026-03-18 16:37</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>@Felix #exercise_feedback 已记录，今天第2次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Felix #exercise_feedback 做得不错，你这周的执行比较稳定。可以尝试把晚餐后活动固定下来，关注空腹和餐后血糖变化。</t>
         </is>
       </c>
     </row>
@@ -1310,14 +1310,14 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>@Felix #exercise_feedback 已记录，今天第3次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Felix #exercise_feedback 今天反馈重点是控糖连续性。建议晚餐主食再略减一些，并保持饭后快走，你有明显进步。</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-03-18 19:43</t>
+          <t>2026-03-18 21:43</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1332,14 +1332,14 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>@Felix #exercise_feedback 已记录，今天第4次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Felix #exercise_feedback 很棒，结合你目前的情况，推荐继续中等强度步行并记录空腹血糖，注意作息规律。</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-03-18 19:46</t>
+          <t>2026-03-18 21:46</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>@Felix #exercise_feedback 已记录，今天第5次反馈：继续保持步数和晚餐控制。</t>
+          <t>@Felix #exercise_feedback 很好。根据你最近的血糖记录，建议餐后再步行10到15分钟，继续保持控糖节奏。</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>收到，谢谢老师，我明天继续打卡。</t>
+          <t>好的，我明天把饭后步行时间再延长一点。</t>
         </is>
       </c>
     </row>

</xml_diff>